<commit_message>
Montaje de reactancia de Neutros
</commit_message>
<xml_diff>
--- a/public/Computos-NP-CC.xlsx
+++ b/public/Computos-NP-CC.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JAraya\Desktop\BESS-JGA\AVANCE DE EQUIPOS MONTADOS\MEJORADA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B32D798-B3A1-4498-9D51-B82FFBA5C7D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DADC329-D646-47F7-BC60-0303CCAC3231}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{43878E65-BAE2-4AD1-A647-97D0F51EE2F0}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{43878E65-BAE2-4AD1-A647-97D0F51EE2F0}"/>
   </bookViews>
   <sheets>
     <sheet name="AvanceJGA" sheetId="3" r:id="rId1"/>
@@ -9480,15 +9480,15 @@
         <v>17</v>
       </c>
       <c r="G244" s="50">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H244" s="50">
         <f t="shared" ref="H244:H248" si="83">E244-G244</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I244" s="51">
         <f t="shared" ref="I244:I248" si="84">IFERROR(G244/E244,"-")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="245" spans="1:9" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Actualizacion de planilla excel
</commit_message>
<xml_diff>
--- a/public/Computos-NP-CC.xlsx
+++ b/public/Computos-NP-CC.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JAraya\Desktop\BESS-JGA\AVANCE DE EQUIPOS MONTADOS\MEJORADA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDC35CC8-2F8E-4E65-80EE-DF0289BECFBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB15161C-B20B-48AD-80CF-9BFC9E76E077}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{43878E65-BAE2-4AD1-A647-97D0F51EE2F0}"/>
   </bookViews>
@@ -3342,15 +3342,15 @@
         <v>17</v>
       </c>
       <c r="G46" s="50">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H46" s="50">
         <f t="shared" si="13"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I46" s="51">
         <f t="shared" si="14"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
@@ -3652,15 +3652,15 @@
         <v>17</v>
       </c>
       <c r="G56" s="50">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H56" s="50">
         <f t="shared" si="16"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I56" s="54">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.25">
@@ -3962,15 +3962,15 @@
         <v>17</v>
       </c>
       <c r="G66" s="50">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H66" s="50">
         <f t="shared" si="19"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I66" s="54">
         <f t="shared" si="20"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.25">
@@ -6752,15 +6752,15 @@
         <v>17</v>
       </c>
       <c r="G156" s="50">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H156" s="50">
         <f t="shared" si="46"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I156" s="54">
         <f t="shared" si="47"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="157" spans="1:9" x14ac:dyDescent="0.25">
@@ -7062,15 +7062,15 @@
         <v>17</v>
       </c>
       <c r="G166" s="50">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H166" s="50">
         <f t="shared" si="49"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I166" s="54">
         <f t="shared" si="50"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="167" spans="1:9" x14ac:dyDescent="0.25">
@@ -7372,15 +7372,15 @@
         <v>17</v>
       </c>
       <c r="G176" s="50">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H176" s="50">
         <f t="shared" si="53"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I176" s="54">
         <f t="shared" si="54"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="177" spans="1:9" x14ac:dyDescent="0.25">
@@ -8736,15 +8736,15 @@
         <v>17</v>
       </c>
       <c r="G220" s="50">
-        <v>96</v>
+        <v>192</v>
       </c>
       <c r="H220" s="50">
         <f t="shared" si="70"/>
-        <v>96</v>
+        <v>0</v>
       </c>
       <c r="I220" s="51">
         <f t="shared" ref="I220:I222" si="72">IFERROR(G220/E220,"-")</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="221" spans="1:9" x14ac:dyDescent="0.25">
@@ -8767,15 +8767,15 @@
         <v>17</v>
       </c>
       <c r="G221" s="50">
-        <v>0</v>
+        <v>192</v>
       </c>
       <c r="H221" s="50">
         <f t="shared" ref="H221:H222" si="73">E221-G221</f>
-        <v>288</v>
+        <v>96</v>
       </c>
       <c r="I221" s="51">
         <f t="shared" si="72"/>
-        <v>0</v>
+        <v>0.66666666666666663</v>
       </c>
     </row>
     <row r="222" spans="1:9" x14ac:dyDescent="0.25">
@@ -9046,15 +9046,15 @@
         <v>17</v>
       </c>
       <c r="G230" s="50">
-        <v>96</v>
+        <v>192</v>
       </c>
       <c r="H230" s="50">
         <f t="shared" si="74"/>
-        <v>96</v>
+        <v>0</v>
       </c>
       <c r="I230" s="51">
         <f t="shared" si="75"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="231" spans="1:9" x14ac:dyDescent="0.25">
@@ -9077,14 +9077,14 @@
         <v>17</v>
       </c>
       <c r="G231" s="50">
-        <v>0</v>
+        <v>192</v>
       </c>
       <c r="H231" s="50">
         <v>288</v>
       </c>
       <c r="I231" s="51">
         <f t="shared" si="75"/>
-        <v>0</v>
+        <v>0.66666666666666663</v>
       </c>
     </row>
     <row r="232" spans="1:9" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Actualizacion de excel + SPDA
</commit_message>
<xml_diff>
--- a/public/Computos-NP-CC.xlsx
+++ b/public/Computos-NP-CC.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JAraya\Desktop\BESS-JGA\AVANCE DE EQUIPOS MONTADOS\MEJORADA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB15161C-B20B-48AD-80CF-9BFC9E76E077}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D90EEC1-73FB-42E9-A14D-0BACAD808645}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{43878E65-BAE2-4AD1-A647-97D0F51EE2F0}"/>
   </bookViews>
@@ -88,7 +88,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1648" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1653" uniqueCount="180">
   <si>
     <t>Seguimiento de cantidades Instaladas en Obra - Nuevo Puerto</t>
   </si>
@@ -625,6 +625,9 @@
   </si>
   <si>
     <t>Montaje de tablero Seccional</t>
+  </si>
+  <si>
+    <t>Montaje mastiles pararrayos</t>
   </si>
 </sst>
 </file>
@@ -1614,8 +1617,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C116F8EF-FEEE-4EAD-838F-B84C8289B566}" name="Tabla1" displayName="Tabla1" ref="A2:I256" totalsRowShown="0" headerRowDxfId="11">
-  <autoFilter ref="A2:I256" xr:uid="{C116F8EF-FEEE-4EAD-838F-B84C8289B566}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C116F8EF-FEEE-4EAD-838F-B84C8289B566}" name="Tabla1" displayName="Tabla1" ref="A2:I257" totalsRowShown="0" headerRowDxfId="11">
+  <autoFilter ref="A2:I257" xr:uid="{C116F8EF-FEEE-4EAD-838F-B84C8289B566}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{EFF3B391-2F8E-4113-91F3-86C7C18FA5B7}" name="Sistema"/>
     <tableColumn id="2" xr3:uid="{C536F8CE-AF56-4C57-9728-3764474816C5}" name="DISCIPLINA"/>
@@ -1932,10 +1935,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6EDF09D0-12EB-42DF-BFFD-4CF2C94E7E96}">
-  <dimension ref="A1:I256"/>
+  <dimension ref="A1:I257"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="35.28515625" customWidth="1"/>
+    <col min="1" max="1" width="38.28515625" customWidth="1"/>
     <col min="2" max="2" width="21.140625" customWidth="1"/>
     <col min="3" max="3" width="20.5703125" customWidth="1"/>
     <col min="4" max="4" width="45.7109375" customWidth="1"/>
@@ -2227,15 +2230,15 @@
         <v>17</v>
       </c>
       <c r="G10" s="50">
-        <v>96</v>
+        <v>192</v>
       </c>
       <c r="H10" s="50">
         <f t="shared" si="0"/>
-        <v>96</v>
+        <v>0</v>
       </c>
       <c r="I10" s="51">
         <f t="shared" si="1"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
@@ -2258,15 +2261,15 @@
         <v>17</v>
       </c>
       <c r="G11" s="50">
-        <v>144</v>
+        <v>288</v>
       </c>
       <c r="H11" s="50">
         <f t="shared" si="0"/>
-        <v>144</v>
+        <v>0</v>
       </c>
       <c r="I11" s="51">
         <f t="shared" si="1"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
@@ -2537,15 +2540,15 @@
         <v>17</v>
       </c>
       <c r="G20" s="50">
-        <v>96</v>
+        <v>192</v>
       </c>
       <c r="H20" s="50">
         <f t="shared" si="4"/>
-        <v>96</v>
+        <v>0</v>
       </c>
       <c r="I20" s="51">
         <f t="shared" si="5"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
@@ -2568,14 +2571,14 @@
         <v>17</v>
       </c>
       <c r="G21" s="50">
-        <v>144</v>
+        <v>288</v>
       </c>
       <c r="H21" s="50">
         <v>144</v>
       </c>
       <c r="I21" s="51">
         <f t="shared" si="5"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
@@ -2846,15 +2849,15 @@
         <v>17</v>
       </c>
       <c r="G30" s="50">
-        <v>96</v>
+        <v>192</v>
       </c>
       <c r="H30" s="50">
         <f t="shared" si="7"/>
-        <v>96</v>
+        <v>0</v>
       </c>
       <c r="I30" s="51">
         <f t="shared" ref="I30:I32" si="9">IFERROR(G30/E30,"-")</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
@@ -2877,15 +2880,15 @@
         <v>17</v>
       </c>
       <c r="G31" s="50">
-        <v>144</v>
+        <v>288</v>
       </c>
       <c r="H31" s="50">
         <f t="shared" si="7"/>
-        <v>144</v>
+        <v>0</v>
       </c>
       <c r="I31" s="51">
         <f t="shared" si="9"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
@@ -3156,15 +3159,15 @@
         <v>17</v>
       </c>
       <c r="G40" s="50">
-        <v>96</v>
+        <v>192</v>
       </c>
       <c r="H40" s="50">
         <f t="shared" si="10"/>
-        <v>96</v>
+        <v>0</v>
       </c>
       <c r="I40" s="51">
         <f t="shared" ref="I40:I42" si="12">IFERROR(G40/E40,"-")</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
@@ -3187,15 +3190,15 @@
         <v>17</v>
       </c>
       <c r="G41" s="50">
-        <v>144</v>
+        <v>288</v>
       </c>
       <c r="H41" s="50">
         <f t="shared" si="10"/>
-        <v>144</v>
+        <v>0</v>
       </c>
       <c r="I41" s="51">
         <f t="shared" si="12"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
@@ -3466,15 +3469,15 @@
         <v>17</v>
       </c>
       <c r="G50" s="50">
-        <v>96</v>
+        <v>192</v>
       </c>
       <c r="H50" s="50">
         <f t="shared" si="13"/>
-        <v>96</v>
+        <v>0</v>
       </c>
       <c r="I50" s="51">
         <f t="shared" ref="I50:I52" si="15">IFERROR(G50/E50,"-")</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
@@ -3497,15 +3500,15 @@
         <v>17</v>
       </c>
       <c r="G51" s="50">
-        <v>144</v>
+        <v>288</v>
       </c>
       <c r="H51" s="50">
         <f t="shared" si="13"/>
-        <v>144</v>
+        <v>0</v>
       </c>
       <c r="I51" s="51">
         <f t="shared" si="15"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.25">
@@ -3776,15 +3779,15 @@
         <v>17</v>
       </c>
       <c r="G60" s="50">
-        <v>96</v>
+        <v>192</v>
       </c>
       <c r="H60" s="50">
         <f t="shared" si="16"/>
-        <v>96</v>
+        <v>0</v>
       </c>
       <c r="I60" s="51">
         <f t="shared" ref="I60:I62" si="18">IFERROR(G60/E60,"-")</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.25">
@@ -3807,15 +3810,15 @@
         <v>17</v>
       </c>
       <c r="G61" s="50">
-        <v>144</v>
+        <v>288</v>
       </c>
       <c r="H61" s="50">
         <f t="shared" si="16"/>
-        <v>144</v>
+        <v>0</v>
       </c>
       <c r="I61" s="51">
         <f t="shared" si="18"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
@@ -5357,15 +5360,15 @@
         <v>17</v>
       </c>
       <c r="G111" s="50">
-        <v>0</v>
+        <v>72</v>
       </c>
       <c r="H111" s="50">
         <f t="shared" ref="H111:H112" si="30">E111-G111</f>
-        <v>144</v>
+        <v>72</v>
       </c>
       <c r="I111" s="51">
         <f t="shared" si="29"/>
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="112" spans="1:9" x14ac:dyDescent="0.25">
@@ -5636,15 +5639,15 @@
         <v>17</v>
       </c>
       <c r="G120" s="50">
-        <v>96</v>
+        <v>192</v>
       </c>
       <c r="H120" s="50">
         <f t="shared" si="31"/>
-        <v>96</v>
+        <v>0</v>
       </c>
       <c r="I120" s="51">
         <f t="shared" ref="I120:I122" si="33">IFERROR(G120/E120,"-")</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="121" spans="1:9" x14ac:dyDescent="0.25">
@@ -5667,15 +5670,15 @@
         <v>17</v>
       </c>
       <c r="G121" s="50">
-        <v>144</v>
+        <v>288</v>
       </c>
       <c r="H121" s="50">
         <f t="shared" ref="H121:H122" si="34">E121-G121</f>
-        <v>144</v>
+        <v>0</v>
       </c>
       <c r="I121" s="51">
         <f t="shared" si="33"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="122" spans="1:9" x14ac:dyDescent="0.25">
@@ -5977,15 +5980,15 @@
         <v>17</v>
       </c>
       <c r="G131" s="50">
-        <v>0</v>
+        <v>288</v>
       </c>
       <c r="H131" s="50">
         <f t="shared" ref="H131:H132" si="38">E131-G131</f>
-        <v>288</v>
+        <v>0</v>
       </c>
       <c r="I131" s="51">
         <f t="shared" si="37"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="132" spans="1:9" x14ac:dyDescent="0.25">
@@ -6287,15 +6290,15 @@
         <v>17</v>
       </c>
       <c r="G141" s="50">
-        <v>144</v>
+        <v>288</v>
       </c>
       <c r="H141" s="50">
         <f t="shared" ref="H141:H142" si="42">E141-G141</f>
-        <v>144</v>
+        <v>0</v>
       </c>
       <c r="I141" s="51">
         <f t="shared" si="41"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="142" spans="1:9" x14ac:dyDescent="0.25">
@@ -6566,15 +6569,15 @@
         <v>17</v>
       </c>
       <c r="G150" s="50">
-        <v>96</v>
+        <v>192</v>
       </c>
       <c r="H150" s="50">
         <f t="shared" si="43"/>
-        <v>96</v>
+        <v>0</v>
       </c>
       <c r="I150" s="51">
         <f t="shared" ref="I150:I152" si="45">IFERROR(G150/E150,"-")</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="151" spans="1:9" x14ac:dyDescent="0.25">
@@ -6597,15 +6600,15 @@
         <v>17</v>
       </c>
       <c r="G151" s="50">
-        <v>144</v>
+        <v>288</v>
       </c>
       <c r="H151" s="50">
         <f t="shared" si="43"/>
-        <v>144</v>
+        <v>0</v>
       </c>
       <c r="I151" s="51">
         <f t="shared" si="45"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="152" spans="1:9" x14ac:dyDescent="0.25">
@@ -6876,15 +6879,15 @@
         <v>17</v>
       </c>
       <c r="G160" s="50">
-        <v>96</v>
+        <v>192</v>
       </c>
       <c r="H160" s="50">
         <f t="shared" si="46"/>
-        <v>96</v>
+        <v>0</v>
       </c>
       <c r="I160" s="51">
         <f t="shared" ref="I160:I162" si="48">IFERROR(G160/E160,"-")</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="161" spans="1:9" x14ac:dyDescent="0.25">
@@ -6938,15 +6941,15 @@
         <v>17</v>
       </c>
       <c r="G162" s="61">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H162" s="61">
         <f t="shared" si="46"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I162" s="62">
         <f t="shared" si="48"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="163" spans="1:9" x14ac:dyDescent="0.25">
@@ -7248,15 +7251,15 @@
         <v>17</v>
       </c>
       <c r="G172" s="61">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H172" s="61">
         <f t="shared" si="52"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I172" s="62">
         <f t="shared" si="51"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="173" spans="1:9" x14ac:dyDescent="0.25">
@@ -7558,15 +7561,15 @@
         <v>17</v>
       </c>
       <c r="G182" s="61">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H182" s="61">
         <f t="shared" si="56"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I182" s="62">
         <f t="shared" si="55"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="183" spans="1:9" x14ac:dyDescent="0.25">
@@ -8426,15 +8429,15 @@
         <v>17</v>
       </c>
       <c r="G210" s="50">
-        <v>96</v>
+        <v>192</v>
       </c>
       <c r="H210" s="50">
         <f t="shared" si="65"/>
-        <v>96</v>
+        <v>0</v>
       </c>
       <c r="I210" s="51">
         <f t="shared" ref="I210" si="67">IFERROR(G210/E210,"-")</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="211" spans="1:9" x14ac:dyDescent="0.25">
@@ -8457,15 +8460,15 @@
         <v>17</v>
       </c>
       <c r="G211" s="50">
-        <v>0</v>
+        <v>288</v>
       </c>
       <c r="H211" s="50">
         <f t="shared" ref="H211:H212" si="68">E211-G211</f>
-        <v>288</v>
+        <v>0</v>
       </c>
       <c r="I211" s="51">
         <f t="shared" ref="I211:I212" si="69">IFERROR(G211/E211,"-")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="212" spans="1:9" x14ac:dyDescent="0.25">
@@ -8767,15 +8770,15 @@
         <v>17</v>
       </c>
       <c r="G221" s="50">
-        <v>192</v>
+        <v>288</v>
       </c>
       <c r="H221" s="50">
         <f t="shared" ref="H221:H222" si="73">E221-G221</f>
-        <v>96</v>
+        <v>0</v>
       </c>
       <c r="I221" s="51">
         <f t="shared" si="72"/>
-        <v>0.66666666666666663</v>
+        <v>1</v>
       </c>
     </row>
     <row r="222" spans="1:9" x14ac:dyDescent="0.25">
@@ -9077,14 +9080,14 @@
         <v>17</v>
       </c>
       <c r="G231" s="50">
-        <v>192</v>
+        <v>288</v>
       </c>
       <c r="H231" s="50">
         <v>288</v>
       </c>
       <c r="I231" s="51">
         <f t="shared" si="75"/>
-        <v>0.66666666666666663</v>
+        <v>1</v>
       </c>
     </row>
     <row r="232" spans="1:9" x14ac:dyDescent="0.25">
@@ -9727,15 +9730,15 @@
         <v>17</v>
       </c>
       <c r="G252" s="49">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H252" s="50">
         <f t="shared" ref="H252" si="89">E252-G252</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I252" s="51">
         <f t="shared" ref="I252" si="90">IFERROR(G252/E252,"-")</f>
-        <v>0.66666666666666663</v>
+        <v>1</v>
       </c>
     </row>
     <row r="253" spans="1:9" x14ac:dyDescent="0.25">
@@ -9836,7 +9839,7 @@
         <v>114</v>
       </c>
       <c r="B256" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C256" t="s">
         <v>94</v>
@@ -9860,6 +9863,37 @@
       <c r="I256" s="51">
         <f t="shared" si="88"/>
         <v>0.5</v>
+      </c>
+    </row>
+    <row r="257" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A257" t="s">
+        <v>114</v>
+      </c>
+      <c r="B257" t="s">
+        <v>71</v>
+      </c>
+      <c r="C257" t="s">
+        <v>94</v>
+      </c>
+      <c r="D257" t="s">
+        <v>179</v>
+      </c>
+      <c r="E257" s="49">
+        <v>3</v>
+      </c>
+      <c r="F257" s="50" t="s">
+        <v>17</v>
+      </c>
+      <c r="G257" s="49">
+        <v>3</v>
+      </c>
+      <c r="H257" s="50">
+        <f t="shared" ref="H257" si="93">E257-G257</f>
+        <v>0</v>
+      </c>
+      <c r="I257" s="51">
+        <f t="shared" ref="I257" si="94">IFERROR(G257/E257,"-")</f>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -9867,7 +9901,7 @@
     <mergeCell ref="B1:I1"/>
   </mergeCells>
   <phoneticPr fontId="10" type="noConversion"/>
-  <conditionalFormatting sqref="I3:I256">
+  <conditionalFormatting sqref="I3:I257">
     <cfRule type="dataBar" priority="1">
       <dataBar>
         <cfvo type="num" val="0"/>
@@ -9903,7 +9937,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>I3:I256</xm:sqref>
+          <xm:sqref>I3:I257</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>

</xml_diff>

<commit_message>
Actualizacion con Montaje de TI
</commit_message>
<xml_diff>
--- a/public/Computos-NP-CC.xlsx
+++ b/public/Computos-NP-CC.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JAraya\Desktop\BESS-JGA\AVANCE DE EQUIPOS MONTADOS\MEJORADA\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JAraya\Desktop\BESS-JGA\AVANCE DE EQUIPOS MONTADOS\NUEVO PUERTO\MEJORADA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D90EEC1-73FB-42E9-A14D-0BACAD808645}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E84F00DD-49C3-48AA-B1A7-E6B55E132F90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{43878E65-BAE2-4AD1-A647-97D0F51EE2F0}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{43878E65-BAE2-4AD1-A647-97D0F51EE2F0}"/>
   </bookViews>
   <sheets>
     <sheet name="AvanceJGA" sheetId="3" r:id="rId1"/>
@@ -3035,15 +3035,15 @@
         <v>17</v>
       </c>
       <c r="G36" s="50">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H36" s="50">
         <f t="shared" si="10"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I36" s="51">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
@@ -9389,15 +9389,15 @@
         <v>17</v>
       </c>
       <c r="G241" s="50">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H241" s="50">
         <f t="shared" si="77"/>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I241" s="51">
         <f t="shared" si="78"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="242" spans="1:9" x14ac:dyDescent="0.25">
@@ -9575,15 +9575,15 @@
         <v>17</v>
       </c>
       <c r="G247" s="50">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H247" s="50">
         <f t="shared" si="83"/>
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="I247" s="51">
         <f t="shared" si="84"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="248" spans="1:9" x14ac:dyDescent="0.25">
@@ -11000,15 +11000,15 @@
         <v>131</v>
       </c>
       <c r="E39" s="65">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F39" s="66">
         <f>'PUNTAS MT'!$C39-'PUNTAS MT'!$E39</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G39" s="67">
         <f>'PUNTAS MT'!$E39/'PUNTAS MT'!$C39</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H39" s="55"/>
       <c r="I39" s="55"/>
@@ -11372,15 +11372,15 @@
       <c r="D54" s="70"/>
       <c r="E54" s="70">
         <f>SUM(E2:E53)</f>
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="F54" s="70">
         <f>SUM(F2:F53)</f>
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="G54" s="71">
         <f>'PUNTAS MT'!$E$54/'PUNTAS MT'!$C$54</f>
-        <v>0.48484848484848486</v>
+        <v>0.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualizacion de puntas BT
</commit_message>
<xml_diff>
--- a/public/Computos-NP-CC.xlsx
+++ b/public/Computos-NP-CC.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JAraya\Desktop\BESS-JGA\AVANCE DE EQUIPOS MONTADOS\NUEVO PUERTO\MEJORADA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15243FE8-F458-44E6-BCF9-D95B3C3C9BE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AAFBCDF-6F62-48E8-A9BC-15949806BCA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{43878E65-BAE2-4AD1-A647-97D0F51EE2F0}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{43878E65-BAE2-4AD1-A647-97D0F51EE2F0}"/>
   </bookViews>
   <sheets>
     <sheet name="AvanceJGA" sheetId="3" r:id="rId1"/>
@@ -1322,6 +1322,12 @@
   </cellStyles>
   <dxfs count="12">
     <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <fill>
         <patternFill patternType="none">
           <bgColor auto="1"/>
@@ -1423,12 +1429,6 @@
           <bgColor theme="4"/>
         </patternFill>
       </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
@@ -1617,20 +1617,14 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C116F8EF-FEEE-4EAD-838F-B84C8289B566}" name="Tabla1" displayName="Tabla1" ref="A2:I257" totalsRowShown="0" headerRowDxfId="11">
-  <autoFilter ref="A2:I257" xr:uid="{C116F8EF-FEEE-4EAD-838F-B84C8289B566}">
-    <filterColumn colId="3">
-      <filters>
-        <filter val="Fundacion Tablero Seccional"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C116F8EF-FEEE-4EAD-838F-B84C8289B566}" name="Tabla1" displayName="Tabla1" ref="A2:I257" totalsRowShown="0" headerRowDxfId="1">
+  <autoFilter ref="A2:I257" xr:uid="{C116F8EF-FEEE-4EAD-838F-B84C8289B566}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{EFF3B391-2F8E-4113-91F3-86C7C18FA5B7}" name="Sistema"/>
     <tableColumn id="2" xr3:uid="{C536F8CE-AF56-4C57-9728-3764474816C5}" name="DISCIPLINA"/>
     <tableColumn id="3" xr3:uid="{B5BAB0E3-FA41-460C-808A-FBDB75C17F64}" name="Area/Sector"/>
     <tableColumn id="4" xr3:uid="{21DA1565-7505-4FFA-9D05-091CE097E902}" name="Tarea"/>
-    <tableColumn id="5" xr3:uid="{CC4898A5-3EC6-4642-897F-54EDBCCE01FF}" name="Cantidad Objetivo" dataDxfId="10"/>
+    <tableColumn id="5" xr3:uid="{CC4898A5-3EC6-4642-897F-54EDBCCE01FF}" name="Cantidad Objetivo" dataDxfId="0"/>
     <tableColumn id="6" xr3:uid="{4580D0A1-48A3-47F7-93E1-8A0C184FED27}" name="Unidad de Medida"/>
     <tableColumn id="7" xr3:uid="{5D6A1260-BD38-46B6-9AF2-875C2F957B23}" name="Ejecutado"/>
     <tableColumn id="8" xr3:uid="{460E4CCD-D08B-47B3-AB8E-BDBEDBE36F2F}" name="Pendiente"/>
@@ -1641,16 +1635,16 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{13657596-22CA-41DC-8732-02E7394DA463}" name="Tabla3" displayName="Tabla3" ref="A1:G54" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8" tableBorderDxfId="7">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{13657596-22CA-41DC-8732-02E7394DA463}" name="Tabla3" displayName="Tabla3" ref="A1:G54" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10" tableBorderDxfId="9">
   <autoFilter ref="A1:G54" xr:uid="{13657596-22CA-41DC-8732-02E7394DA463}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{56C0A5E9-A046-4527-A482-E4840ADAC2D0}" name="Descripcion de Tarea" dataDxfId="6"/>
-    <tableColumn id="2" xr3:uid="{E90C49B1-5769-4E3B-B661-60B1F550D9B8}" name="Power Block" dataDxfId="5"/>
-    <tableColumn id="3" xr3:uid="{F3853004-6657-4249-9BB7-E96901BAB015}" name="Objetivo" dataDxfId="4"/>
-    <tableColumn id="4" xr3:uid="{B31C1388-6D2A-427E-B72C-E636DC131876}" name="Formacion" dataDxfId="3"/>
-    <tableColumn id="5" xr3:uid="{DB58243E-7754-4863-A6B4-8F10F25C948D}" name="Ejecutado" dataDxfId="2"/>
-    <tableColumn id="6" xr3:uid="{2E25E639-4B45-400F-908F-0A958665D8DA}" name="Restante" dataDxfId="1"/>
-    <tableColumn id="7" xr3:uid="{1F70A694-3F5D-499B-B682-2922AC1C4522}" name="Avance" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{56C0A5E9-A046-4527-A482-E4840ADAC2D0}" name="Descripcion de Tarea" dataDxfId="8"/>
+    <tableColumn id="2" xr3:uid="{E90C49B1-5769-4E3B-B661-60B1F550D9B8}" name="Power Block" dataDxfId="7"/>
+    <tableColumn id="3" xr3:uid="{F3853004-6657-4249-9BB7-E96901BAB015}" name="Objetivo" dataDxfId="6"/>
+    <tableColumn id="4" xr3:uid="{B31C1388-6D2A-427E-B72C-E636DC131876}" name="Formacion" dataDxfId="5"/>
+    <tableColumn id="5" xr3:uid="{DB58243E-7754-4863-A6B4-8F10F25C948D}" name="Ejecutado" dataDxfId="4"/>
+    <tableColumn id="6" xr3:uid="{2E25E639-4B45-400F-908F-0A958665D8DA}" name="Restante" dataDxfId="3"/>
+    <tableColumn id="7" xr3:uid="{1F70A694-3F5D-499B-B682-2922AC1C4522}" name="Avance" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1946,7 +1940,7 @@
   <cols>
     <col min="1" max="1" width="38.28515625" customWidth="1"/>
     <col min="2" max="2" width="21.140625" customWidth="1"/>
-    <col min="3" max="3" width="20.5703125" customWidth="1"/>
+    <col min="3" max="3" width="17.5703125" customWidth="1"/>
     <col min="4" max="4" width="45.7109375" customWidth="1"/>
     <col min="5" max="5" width="15.5703125" style="49" customWidth="1"/>
     <col min="6" max="7" width="15" customWidth="1"/>
@@ -1999,7 +1993,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="3" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>112</v>
       </c>
@@ -2030,7 +2024,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>112</v>
       </c>
@@ -2061,7 +2055,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>112</v>
       </c>
@@ -2123,7 +2117,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>112</v>
       </c>
@@ -2154,7 +2148,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>112</v>
       </c>
@@ -2185,7 +2179,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>112</v>
       </c>
@@ -2216,7 +2210,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>112</v>
       </c>
@@ -2247,7 +2241,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>112</v>
       </c>
@@ -2278,7 +2272,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="60" t="s">
         <v>112</v>
       </c>
@@ -2309,7 +2303,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="12.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>112</v>
       </c>
@@ -2340,7 +2334,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>112</v>
       </c>
@@ -2371,7 +2365,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>112</v>
       </c>
@@ -2433,7 +2427,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>112</v>
       </c>
@@ -2464,7 +2458,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>112</v>
       </c>
@@ -2495,7 +2489,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>112</v>
       </c>
@@ -2526,7 +2520,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>112</v>
       </c>
@@ -2557,7 +2551,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>112</v>
       </c>
@@ -2587,7 +2581,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="60" t="s">
         <v>112</v>
       </c>
@@ -2618,7 +2612,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>112</v>
       </c>
@@ -2649,7 +2643,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>112</v>
       </c>
@@ -2680,7 +2674,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>112</v>
       </c>
@@ -2742,7 +2736,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>112</v>
       </c>
@@ -2773,7 +2767,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>112</v>
       </c>
@@ -2804,7 +2798,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>112</v>
       </c>
@@ -2835,7 +2829,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>112</v>
       </c>
@@ -2866,7 +2860,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>112</v>
       </c>
@@ -2897,7 +2891,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="60" t="s">
         <v>112</v>
       </c>
@@ -2928,7 +2922,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>112</v>
       </c>
@@ -2959,7 +2953,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>112</v>
       </c>
@@ -2990,7 +2984,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>112</v>
       </c>
@@ -3052,7 +3046,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>112</v>
       </c>
@@ -3083,7 +3077,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>112</v>
       </c>
@@ -3114,7 +3108,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>112</v>
       </c>
@@ -3145,7 +3139,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>112</v>
       </c>
@@ -3176,7 +3170,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>112</v>
       </c>
@@ -3207,7 +3201,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" s="60" t="s">
         <v>112</v>
       </c>
@@ -3227,18 +3221,18 @@
         <v>17</v>
       </c>
       <c r="G42" s="61">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H42" s="61">
         <f t="shared" si="10"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I42" s="62">
         <f t="shared" si="12"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>112</v>
       </c>
@@ -3269,7 +3263,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>112</v>
       </c>
@@ -3300,7 +3294,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>112</v>
       </c>
@@ -3362,7 +3356,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="47" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>112</v>
       </c>
@@ -3393,7 +3387,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>112</v>
       </c>
@@ -3424,7 +3418,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>112</v>
       </c>
@@ -3455,7 +3449,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>112</v>
       </c>
@@ -3486,7 +3480,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>112</v>
       </c>
@@ -3517,7 +3511,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="52" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52" s="60" t="s">
         <v>112</v>
       </c>
@@ -3537,18 +3531,18 @@
         <v>17</v>
       </c>
       <c r="G52" s="61">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H52" s="61">
         <f t="shared" si="13"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I52" s="62">
         <f t="shared" si="15"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>112</v>
       </c>
@@ -3579,7 +3573,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>112</v>
       </c>
@@ -3610,7 +3604,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>112</v>
       </c>
@@ -3672,7 +3666,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="57" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>112</v>
       </c>
@@ -3703,7 +3697,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="58" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>112</v>
       </c>
@@ -3734,7 +3728,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="59" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>112</v>
       </c>
@@ -3765,7 +3759,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="60" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>112</v>
       </c>
@@ -3796,7 +3790,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="61" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>112</v>
       </c>
@@ -3827,7 +3821,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A62" s="60" t="s">
         <v>112</v>
       </c>
@@ -3847,18 +3841,18 @@
         <v>17</v>
       </c>
       <c r="G62" s="61">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H62" s="61">
         <f t="shared" si="16"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I62" s="62">
         <f t="shared" si="18"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="63" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="63" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>112</v>
       </c>
@@ -3889,7 +3883,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>112</v>
       </c>
@@ -3920,7 +3914,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="65" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>112</v>
       </c>
@@ -3982,7 +3976,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="67" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>112</v>
       </c>
@@ -4013,7 +4007,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="68" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>112</v>
       </c>
@@ -4044,7 +4038,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="69" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>112</v>
       </c>
@@ -4075,7 +4069,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="70" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>112</v>
       </c>
@@ -4106,7 +4100,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="71" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>112</v>
       </c>
@@ -4137,7 +4131,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="72" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A72" s="60" t="s">
         <v>112</v>
       </c>
@@ -4157,18 +4151,18 @@
         <v>17</v>
       </c>
       <c r="G72" s="61">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H72" s="61">
         <f t="shared" si="19"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I72" s="62">
         <f t="shared" si="20"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="73" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="73" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>112</v>
       </c>
@@ -4199,7 +4193,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="74" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>112</v>
       </c>
@@ -4230,7 +4224,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="75" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>112</v>
       </c>
@@ -4292,7 +4286,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="77" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>112</v>
       </c>
@@ -4323,7 +4317,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="78" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>112</v>
       </c>
@@ -4354,7 +4348,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="79" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>112</v>
       </c>
@@ -4385,7 +4379,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="80" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>112</v>
       </c>
@@ -4416,7 +4410,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="81" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>112</v>
       </c>
@@ -4447,7 +4441,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="82" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A82" s="60" t="s">
         <v>112</v>
       </c>
@@ -4478,7 +4472,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="83" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>112</v>
       </c>
@@ -4509,7 +4503,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="84" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>112</v>
       </c>
@@ -4540,7 +4534,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="85" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>112</v>
       </c>
@@ -4602,7 +4596,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="87" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>112</v>
       </c>
@@ -4633,7 +4627,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="88" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>112</v>
       </c>
@@ -4664,7 +4658,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="89" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>112</v>
       </c>
@@ -4695,7 +4689,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="90" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>112</v>
       </c>
@@ -4726,7 +4720,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="91" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>112</v>
       </c>
@@ -4757,7 +4751,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="92" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A92" s="60" t="s">
         <v>112</v>
       </c>
@@ -4788,7 +4782,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="93" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>112</v>
       </c>
@@ -4819,7 +4813,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="94" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>112</v>
       </c>
@@ -4850,7 +4844,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="95" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>112</v>
       </c>
@@ -4912,7 +4906,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="97" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>112</v>
       </c>
@@ -4943,7 +4937,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="98" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>112</v>
       </c>
@@ -4974,7 +4968,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="99" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>112</v>
       </c>
@@ -5005,7 +4999,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="100" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>112</v>
       </c>
@@ -5036,7 +5030,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="101" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>112</v>
       </c>
@@ -5067,7 +5061,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="102" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A102" s="60" t="s">
         <v>112</v>
       </c>
@@ -5098,7 +5092,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="103" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>112</v>
       </c>
@@ -5129,7 +5123,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="104" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>112</v>
       </c>
@@ -5160,7 +5154,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="105" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>112</v>
       </c>
@@ -5222,7 +5216,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>112</v>
       </c>
@@ -5253,7 +5247,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="108" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>112</v>
       </c>
@@ -5284,7 +5278,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="109" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>112</v>
       </c>
@@ -5315,7 +5309,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="110" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>112</v>
       </c>
@@ -5335,18 +5329,18 @@
         <v>17</v>
       </c>
       <c r="G110" s="50">
-        <v>48</v>
+        <v>96</v>
       </c>
       <c r="H110" s="50">
         <f t="shared" si="27"/>
-        <v>48</v>
+        <v>0</v>
       </c>
       <c r="I110" s="51">
         <f t="shared" ref="I110:I112" si="29">IFERROR(G110/E110,"-")</f>
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="111" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="111" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>112</v>
       </c>
@@ -5366,18 +5360,18 @@
         <v>17</v>
       </c>
       <c r="G111" s="50">
-        <v>72</v>
+        <v>144</v>
       </c>
       <c r="H111" s="50">
         <f t="shared" ref="H111:H112" si="30">E111-G111</f>
-        <v>72</v>
+        <v>0</v>
       </c>
       <c r="I111" s="51">
         <f t="shared" si="29"/>
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="112" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="112" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A112" s="60" t="s">
         <v>112</v>
       </c>
@@ -5408,7 +5402,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="113" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>112</v>
       </c>
@@ -5439,7 +5433,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="114" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>112</v>
       </c>
@@ -5470,7 +5464,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="115" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>112</v>
       </c>
@@ -5532,7 +5526,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="117" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>112</v>
       </c>
@@ -5563,7 +5557,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="118" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>112</v>
       </c>
@@ -5594,7 +5588,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="119" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>112</v>
       </c>
@@ -5625,7 +5619,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="120" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>112</v>
       </c>
@@ -5656,7 +5650,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="121" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>112</v>
       </c>
@@ -5687,7 +5681,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="122" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A122" s="60" t="s">
         <v>112</v>
       </c>
@@ -5718,7 +5712,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="123" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>112</v>
       </c>
@@ -5749,7 +5743,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="124" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>112</v>
       </c>
@@ -5780,7 +5774,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="125" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>112</v>
       </c>
@@ -5842,7 +5836,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="127" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>112</v>
       </c>
@@ -5873,7 +5867,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="128" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>112</v>
       </c>
@@ -5904,7 +5898,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="129" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>112</v>
       </c>
@@ -5935,7 +5929,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="130" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>112</v>
       </c>
@@ -5966,7 +5960,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="131" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>112</v>
       </c>
@@ -5997,7 +5991,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="132" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A132" s="60" t="s">
         <v>112</v>
       </c>
@@ -6028,7 +6022,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="133" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>112</v>
       </c>
@@ -6059,7 +6053,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="134" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>112</v>
       </c>
@@ -6090,7 +6084,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="135" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
         <v>112</v>
       </c>
@@ -6152,7 +6146,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="137" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
         <v>112</v>
       </c>
@@ -6183,7 +6177,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="138" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
         <v>112</v>
       </c>
@@ -6214,7 +6208,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="139" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>112</v>
       </c>
@@ -6245,7 +6239,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="140" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
         <v>112</v>
       </c>
@@ -6276,7 +6270,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="141" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
         <v>112</v>
       </c>
@@ -6307,7 +6301,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="142" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A142" s="60" t="s">
         <v>112</v>
       </c>
@@ -6338,7 +6332,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="143" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
         <v>112</v>
       </c>
@@ -6369,7 +6363,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="144" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
         <v>112</v>
       </c>
@@ -6400,7 +6394,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="145" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
         <v>112</v>
       </c>
@@ -6462,7 +6456,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="147" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
         <v>112</v>
       </c>
@@ -6493,7 +6487,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="148" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
         <v>112</v>
       </c>
@@ -6524,7 +6518,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="149" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
         <v>112</v>
       </c>
@@ -6555,7 +6549,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="150" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
         <v>112</v>
       </c>
@@ -6586,7 +6580,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="151" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
         <v>112</v>
       </c>
@@ -6617,7 +6611,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="152" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A152" s="60" t="s">
         <v>112</v>
       </c>
@@ -6648,7 +6642,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="153" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
         <v>112</v>
       </c>
@@ -6679,7 +6673,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="154" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
         <v>112</v>
       </c>
@@ -6710,7 +6704,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="155" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
         <v>112</v>
       </c>
@@ -6772,7 +6766,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="157" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
         <v>112</v>
       </c>
@@ -6803,7 +6797,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="158" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
         <v>112</v>
       </c>
@@ -6834,7 +6828,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="159" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
         <v>112</v>
       </c>
@@ -6865,7 +6859,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="160" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
         <v>112</v>
       </c>
@@ -6896,7 +6890,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="161" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
         <v>112</v>
       </c>
@@ -6927,7 +6921,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="162" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A162" s="60" t="s">
         <v>112</v>
       </c>
@@ -6958,7 +6952,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="163" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
         <v>112</v>
       </c>
@@ -6989,7 +6983,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="164" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
         <v>112</v>
       </c>
@@ -7020,7 +7014,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="165" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
         <v>112</v>
       </c>
@@ -7082,7 +7076,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="167" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
         <v>112</v>
       </c>
@@ -7113,7 +7107,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="168" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
         <v>112</v>
       </c>
@@ -7144,7 +7138,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="169" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
         <v>112</v>
       </c>
@@ -7175,7 +7169,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="170" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
         <v>112</v>
       </c>
@@ -7206,7 +7200,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="171" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
         <v>112</v>
       </c>
@@ -7237,7 +7231,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="172" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A172" s="60" t="s">
         <v>112</v>
       </c>
@@ -7268,7 +7262,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="173" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
         <v>112</v>
       </c>
@@ -7299,7 +7293,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="174" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
         <v>112</v>
       </c>
@@ -7330,7 +7324,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="175" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
         <v>112</v>
       </c>
@@ -7392,7 +7386,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="177" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
         <v>112</v>
       </c>
@@ -7423,7 +7417,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="178" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
         <v>112</v>
       </c>
@@ -7454,7 +7448,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="179" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
         <v>112</v>
       </c>
@@ -7485,7 +7479,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="180" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
         <v>112</v>
       </c>
@@ -7516,7 +7510,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="181" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
         <v>112</v>
       </c>
@@ -7547,7 +7541,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="182" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A182" s="60" t="s">
         <v>112</v>
       </c>
@@ -7578,7 +7572,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="183" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
         <v>112</v>
       </c>
@@ -7609,7 +7603,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="184" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
         <v>112</v>
       </c>
@@ -7640,7 +7634,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="185" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
         <v>112</v>
       </c>
@@ -7702,7 +7696,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="187" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
         <v>112</v>
       </c>
@@ -7733,7 +7727,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="188" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
         <v>112</v>
       </c>
@@ -7764,7 +7758,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="189" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
         <v>112</v>
       </c>
@@ -7795,7 +7789,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="190" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
         <v>112</v>
       </c>
@@ -7826,7 +7820,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="191" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
         <v>112</v>
       </c>
@@ -7857,7 +7851,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="192" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A192" s="60" t="s">
         <v>112</v>
       </c>
@@ -7888,7 +7882,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="193" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
         <v>112</v>
       </c>
@@ -7919,7 +7913,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="194" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
         <v>112</v>
       </c>
@@ -7950,7 +7944,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="195" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
         <v>112</v>
       </c>
@@ -8012,7 +8006,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="197" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
         <v>112</v>
       </c>
@@ -8043,7 +8037,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="198" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
         <v>112</v>
       </c>
@@ -8074,7 +8068,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="199" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
         <v>112</v>
       </c>
@@ -8105,7 +8099,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="200" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
         <v>112</v>
       </c>
@@ -8136,7 +8130,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="201" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A201" t="s">
         <v>112</v>
       </c>
@@ -8167,7 +8161,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="202" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A202" s="60" t="s">
         <v>112</v>
       </c>
@@ -8198,7 +8192,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="203" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
         <v>112</v>
       </c>
@@ -8229,7 +8223,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="204" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A204" t="s">
         <v>112</v>
       </c>
@@ -8260,7 +8254,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="205" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
         <v>112</v>
       </c>
@@ -8322,7 +8316,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="207" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
         <v>112</v>
       </c>
@@ -8353,7 +8347,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="208" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
         <v>112</v>
       </c>
@@ -8384,7 +8378,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="209" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A209" t="s">
         <v>112</v>
       </c>
@@ -8415,7 +8409,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="210" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A210" t="s">
         <v>112</v>
       </c>
@@ -8446,7 +8440,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="211" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A211" t="s">
         <v>112</v>
       </c>
@@ -8477,7 +8471,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="212" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A212" s="60" t="s">
         <v>112</v>
       </c>
@@ -8508,7 +8502,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="213" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A213" t="s">
         <v>112</v>
       </c>
@@ -8539,7 +8533,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="214" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A214" t="s">
         <v>112</v>
       </c>
@@ -8570,7 +8564,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="215" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
         <v>112</v>
       </c>
@@ -8632,7 +8626,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="217" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A217" t="s">
         <v>112</v>
       </c>
@@ -8663,7 +8657,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="218" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A218" t="s">
         <v>112</v>
       </c>
@@ -8694,7 +8688,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="219" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A219" t="s">
         <v>112</v>
       </c>
@@ -8725,7 +8719,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="220" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A220" t="s">
         <v>112</v>
       </c>
@@ -8756,7 +8750,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="221" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A221" t="s">
         <v>112</v>
       </c>
@@ -8787,7 +8781,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="222" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A222" s="60" t="s">
         <v>112</v>
       </c>
@@ -8818,7 +8812,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="223" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A223" t="s">
         <v>112</v>
       </c>
@@ -8849,7 +8843,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="224" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A224" t="s">
         <v>112</v>
       </c>
@@ -8880,7 +8874,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="225" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A225" t="s">
         <v>112</v>
       </c>
@@ -8942,7 +8936,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="227" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A227" t="s">
         <v>112</v>
       </c>
@@ -8973,7 +8967,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="228" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A228" t="s">
         <v>112</v>
       </c>
@@ -9004,7 +8998,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="229" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A229" t="s">
         <v>112</v>
       </c>
@@ -9035,7 +9029,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="230" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A230" t="s">
         <v>112</v>
       </c>
@@ -9066,7 +9060,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="231" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A231" t="s">
         <v>112</v>
       </c>
@@ -9096,7 +9090,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="232" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A232" s="60" t="s">
         <v>112</v>
       </c>
@@ -9127,7 +9121,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="233" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A233" t="s">
         <v>113</v>
       </c>
@@ -9158,7 +9152,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="234" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A234" t="s">
         <v>113</v>
       </c>
@@ -9189,7 +9183,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="235" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A235" t="s">
         <v>113</v>
       </c>
@@ -9220,7 +9214,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="236" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A236" t="s">
         <v>113</v>
       </c>
@@ -9251,7 +9245,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="237" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A237" t="s">
         <v>113</v>
       </c>
@@ -9282,7 +9276,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="238" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A238" t="s">
         <v>113</v>
       </c>
@@ -9313,7 +9307,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="239" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A239" t="s">
         <v>113</v>
       </c>
@@ -9344,7 +9338,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="240" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A240" t="s">
         <v>113</v>
       </c>
@@ -9375,7 +9369,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="241" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A241" t="s">
         <v>113</v>
       </c>
@@ -9406,7 +9400,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="242" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A242" t="s">
         <v>113</v>
       </c>
@@ -9437,7 +9431,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="243" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A243" t="s">
         <v>113</v>
       </c>
@@ -9468,7 +9462,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="244" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A244" t="s">
         <v>113</v>
       </c>
@@ -9499,7 +9493,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="245" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A245" t="s">
         <v>113</v>
       </c>
@@ -9530,7 +9524,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="246" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A246" t="s">
         <v>113</v>
       </c>
@@ -9561,7 +9555,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="247" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A247" t="s">
         <v>113</v>
       </c>
@@ -9592,7 +9586,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="248" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A248" t="s">
         <v>113</v>
       </c>
@@ -9623,7 +9617,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="249" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A249" t="s">
         <v>117</v>
       </c>
@@ -9654,7 +9648,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="250" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A250" t="s">
         <v>114</v>
       </c>
@@ -9685,7 +9679,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="251" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A251" t="s">
         <v>114</v>
       </c>
@@ -9716,7 +9710,7 @@
         <v>0.66666666666666663</v>
       </c>
     </row>
-    <row r="252" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A252" t="s">
         <v>114</v>
       </c>
@@ -9747,7 +9741,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="253" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A253" t="s">
         <v>114</v>
       </c>
@@ -9778,7 +9772,7 @@
         <v>0.6</v>
       </c>
     </row>
-    <row r="254" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A254" t="s">
         <v>114</v>
       </c>
@@ -9809,7 +9803,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="255" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A255" t="s">
         <v>114</v>
       </c>
@@ -9840,7 +9834,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="256" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A256" t="s">
         <v>114</v>
       </c>
@@ -9871,7 +9865,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="257" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A257" t="s">
         <v>114</v>
       </c>

</xml_diff>